<commit_message>
H045 v5（5.0.0.0）新增 Extra Bet：2 倍押注、Card-On FG 週期 1/30（NB 的 5 倍）；92A 加 eb_base_game／eb_free_game（FG 卡同 NB、BG 重解）；Simulator bet mode 1、Demogame Extra Bet 按鈕、Help／game_rule 同步（Card-On 驗證進行中）
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Slots/H045_超級鑽石/文件/101015_Help.xlsx
+++ b/Slots/H045_超級鑽石/文件/101015_Help.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I123"/>
+  <dimension ref="A1:I130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1701,7 +1701,7 @@
     <row r="70">
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>BUY FEATURE</t>
+          <t>EXTRA BET</t>
         </is>
       </c>
     </row>
@@ -1738,14 +1738,14 @@
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>購買特色</t>
+          <t>額外投注</t>
         </is>
       </c>
       <c r="E72" s="7" t="n"/>
       <c r="F72" s="8" t="n"/>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>BUY FEATURE</t>
+          <t>EXTRA BET</t>
         </is>
       </c>
       <c r="H72" s="7" t="n"/>
@@ -1762,14 +1762,14 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>▪ 點擊「購買特色」按鈕，將開啟「購買特色」選單。</t>
+          <t>▪ 額外投注的扣款為 {2} × 您所選的基礎投注。</t>
         </is>
       </c>
       <c r="E73" s="7" t="n"/>
       <c r="F73" s="8" t="n"/>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>▪ BY TAPPING ON THE BUY FEATURE BUTTON, YOU WILL OPEN THE BUY FEATURE MENU.</t>
+          <t>▪ EXTRA BET COSTS {2} × THE BASE BET YOU SELECT.</t>
         </is>
       </c>
       <c r="H73" s="7" t="n"/>
@@ -1778,14 +1778,14 @@
     <row r="74">
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>▪ 您可以按「+」或「-」按鈕調整投注額與數量。</t>
+          <t>▪ 所有獎金仍依您所選的基礎投注計算。</t>
         </is>
       </c>
       <c r="E74" s="7" t="n"/>
       <c r="F74" s="8" t="n"/>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>▪ YOU CAN INCREASE OR DECREASE YOUR BET AND QUANTITY BY PRESSING THE "+" OR "-" BUTTONS.</t>
+          <t>▪ ALL WINS ARE STILL CALCULATED ON THE BASE BET YOU SELECT.</t>
         </is>
       </c>
       <c r="H74" s="7" t="n"/>
@@ -1794,94 +1794,91 @@
     <row r="75">
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>▪ 以所選投注額的 {50} 倍購買，直接觸發免費遊戲特色。</t>
+          <t>▪ 免費遊戲的觸發機率提升為一般投注的 {5} 倍。</t>
         </is>
       </c>
       <c r="E75" s="7" t="n"/>
       <c r="F75" s="8" t="n"/>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>▪ THE FREE GAME FEATURE CAN BE TRIGGERED DIRECTLY BY BUYING IT FOR {50}X THE SELECTED BET.</t>
+          <t>▪ THE CHANCE TO TRIGGER THE FREE GAME FEATURE IS {5} TIMES THAT OF THE NORMAL BET.</t>
         </is>
       </c>
       <c r="H75" s="7" t="n"/>
       <c r="I75" s="8" t="n"/>
     </row>
-    <row r="76">
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>▪ 最多可一次購買 {99} 次。</t>
-        </is>
-      </c>
-      <c r="E76" s="7" t="n"/>
-      <c r="F76" s="8" t="n"/>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>▪ THE MAXIMUM SELECTED QUANTITY IS {99}.</t>
-        </is>
-      </c>
-      <c r="H76" s="7" t="n"/>
-      <c r="I76" s="8" t="n"/>
-    </row>
     <row r="77">
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>▪ 總價 = 價格 × 數量，顯示在「購買特色」選單中。</t>
-        </is>
-      </c>
-      <c r="E77" s="7" t="n"/>
-      <c r="F77" s="8" t="n"/>
-      <c r="G77" s="6" t="inlineStr">
-        <is>
-          <t>▪ TOTAL PRICE = PRICE × QUANTITY, WHICH IS DISPLAYED IN THE BUY FEATURE MENU.</t>
-        </is>
-      </c>
-      <c r="H77" s="7" t="n"/>
-      <c r="I77" s="8" t="n"/>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>BUY FEATURE</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>▪ 按下「旋轉」按鈕／「購買並開始遊戲」按鈕後，「購買特色」選單中顯示的價格將從玩家的餘額中扣除。</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="n"/>
-      <c r="F78" s="8" t="n"/>
-      <c r="G78" s="6" t="inlineStr">
-        <is>
-          <t>▪ AFTER PRESSING THE SPIN BUTTON / BUY BUTTON, THE PRICE DISPLAYED IN THE BUY FEATURE MENU IS DEDUCTED FROM THE PLAYER'S BALANCE.</t>
-        </is>
-      </c>
-      <c r="H78" s="7" t="n"/>
-      <c r="I78" s="8" t="n"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>繁中</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>英文</t>
+        </is>
+      </c>
     </row>
     <row r="79">
+      <c r="B79" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>主要標題</t>
+        </is>
+      </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>▪ 第一局之後，玩家需按「旋轉」按鈕逐次進行，或點選「自動旋轉」按鈕自動進行剩餘的「購買特色」；剩餘數量為 {0} 時自動旋轉停止。</t>
+          <t>購買特色</t>
         </is>
       </c>
       <c r="E79" s="7" t="n"/>
       <c r="F79" s="8" t="n"/>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>▪ AFTER THE FIRST GAME, THE PLAYER PRESSES THE SPIN BUTTON TO PLAY EACH REMAINING BUY FEATURE, OR TAPS THE AUTO SPIN BUTTON TO PLAY THEM AUTOMATICALLY. AUTO SPIN STOPS WHEN THE REMAINING QUANTITY IS {0}.</t>
+          <t>BUY FEATURE</t>
         </is>
       </c>
       <c r="H79" s="7" t="n"/>
       <c r="I79" s="8" t="n"/>
     </row>
     <row r="80">
+      <c r="B80" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>規則說明</t>
+        </is>
+      </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>▪ 如果網路中斷／瀏覽器關閉，剩餘的「購買特色」數量將被取消。</t>
+          <t>▪ 點擊「購買特色」按鈕，將開啟「購買特色」選單。</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
       <c r="F80" s="8" t="n"/>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>▪ IN CASE OF NETWORK DISCONNECTION / BROWSER CLOSE, THE REMAINING BUY FEATURE QUANTITY WILL BE CANCELLED.</t>
+          <t>▪ BY TAPPING ON THE BUY FEATURE BUTTON, YOU WILL OPEN THE BUY FEATURE MENU.</t>
         </is>
       </c>
       <c r="H80" s="7" t="n"/>
@@ -1890,14 +1887,14 @@
     <row r="81">
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>▪ 在最後一個「購買特色」完成之前，無法調整投注，也無法取消剩餘的「購買特色」。</t>
+          <t>▪ 您可以按「+」或「-」按鈕調整投注額與數量。</t>
         </is>
       </c>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="8" t="n"/>
       <c r="G81" s="6" t="inlineStr">
         <is>
-          <t>▪ THE BET CANNOT BE ADJUSTED AND THE REMAINING BUY FEATURE CANNOT BE CANCELLED BEFORE THE LAST BUY FEATURE IS COMPLETED.</t>
+          <t>▪ YOU CAN INCREASE OR DECREASE YOUR BET AND QUANTITY BY PRESSING THE "+" OR "-" BUTTONS.</t>
         </is>
       </c>
       <c r="H81" s="7" t="n"/>
@@ -1906,91 +1903,94 @@
     <row r="82">
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>▪ 所有「購買特色」完成後，投注將切換回購買前的投注。</t>
+          <t>▪ 以所選投注額的 {50} 倍購買，直接觸發免費遊戲特色。</t>
         </is>
       </c>
       <c r="E82" s="7" t="n"/>
       <c r="F82" s="8" t="n"/>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>▪ AFTER ALL BUY FEATURE ROUNDS ARE COMPLETED, THE BET WILL SWITCH BACK TO THE BET BEFORE THE PURCHASE.</t>
+          <t>▪ THE FREE GAME FEATURE CAN BE TRIGGERED DIRECTLY BY BUYING IT FOR {50}X THE SELECTED BET.</t>
         </is>
       </c>
       <c r="H82" s="7" t="n"/>
       <c r="I82" s="8" t="n"/>
     </row>
+    <row r="83">
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>▪ 最多可一次購買 {99} 次。</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="n"/>
+      <c r="F83" s="8" t="n"/>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>▪ THE MAXIMUM SELECTED QUANTITY IS {99}.</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="n"/>
+      <c r="I83" s="8" t="n"/>
+    </row>
     <row r="84">
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>OP JACKPOT</t>
-        </is>
-      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>▪ 總價 = 價格 × 數量，顯示在「購買特色」選單中。</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="n"/>
+      <c r="F84" s="8" t="n"/>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>▪ TOTAL PRICE = PRICE × QUANTITY, WHICH IS DISPLAYED IN THE BUY FEATURE MENU.</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="n"/>
+      <c r="I84" s="8" t="n"/>
     </row>
     <row r="85">
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>項目</t>
-        </is>
-      </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>繁中</t>
-        </is>
-      </c>
-      <c r="G85" s="5" t="inlineStr">
-        <is>
-          <t>英文</t>
-        </is>
-      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>▪ 按下「旋轉」按鈕／「購買並開始遊戲」按鈕後，「購買特色」選單中顯示的價格將從玩家的餘額中扣除。</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="n"/>
+      <c r="F85" s="8" t="n"/>
+      <c r="G85" s="6" t="inlineStr">
+        <is>
+          <t>▪ AFTER PRESSING THE SPIN BUTTON / BUY BUTTON, THE PRICE DISPLAYED IN THE BUY FEATURE MENU IS DEDUCTED FROM THE PLAYER'S BALANCE.</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="n"/>
+      <c r="I85" s="8" t="n"/>
     </row>
     <row r="86">
-      <c r="B86" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C86" s="6" t="inlineStr">
-        <is>
-          <t>主要標題</t>
-        </is>
-      </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>OP JACKPOT</t>
+          <t>▪ 第一局之後，玩家需按「旋轉」按鈕逐次進行，或點選「自動旋轉」按鈕自動進行剩餘的「購買特色」；剩餘數量為 {0} 時自動旋轉停止。</t>
         </is>
       </c>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="8" t="n"/>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t>OP JACKPOT</t>
+          <t>▪ AFTER THE FIRST GAME, THE PLAYER PRESSES THE SPIN BUTTON TO PLAY EACH REMAINING BUY FEATURE, OR TAPS THE AUTO SPIN BUTTON TO PLAY THEM AUTOMATICALLY. AUTO SPIN STOPS WHEN THE REMAINING QUANTITY IS {0}.</t>
         </is>
       </c>
       <c r="H86" s="7" t="n"/>
       <c r="I86" s="8" t="n"/>
     </row>
     <row r="87">
-      <c r="B87" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C87" s="6" t="inlineStr">
-        <is>
-          <t>規則說明</t>
-        </is>
-      </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>▪ 在遊戲中，OP JACKPOT 特色由盤面上的 [C1] 隨機觸發。</t>
+          <t>▪ 如果網路中斷／瀏覽器關閉，剩餘的「購買特色」數量將被取消。</t>
         </is>
       </c>
       <c r="E87" s="7" t="n"/>
       <c r="F87" s="8" t="n"/>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>▪ OP JACKPOT FEATURE IS TRIGGERED RANDOMLY BY {1} OR MORE [C1] ON THE REELS.</t>
+          <t>▪ IN CASE OF NETWORK DISCONNECTION / BROWSER CLOSE, THE REMAINING BUY FEATURE QUANTITY WILL BE CANCELLED.</t>
         </is>
       </c>
       <c r="H87" s="7" t="n"/>
@@ -1999,14 +1999,14 @@
     <row r="88">
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>▪ OP JACKPOT 特色會在畫面中出現 {12} 個 [幣]，其中包括 [GRAND]、[MAJOR]、[MINOR] 及 [MINI]。</t>
+          <t>▪ 在最後一個「購買特色」完成之前，無法調整投注，也無法取消剩餘的「購買特色」。</t>
         </is>
       </c>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="8" t="n"/>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>▪ DURING OP JACKPOT FEATURE, THERE ARE {12} [COIN] WHICH CONSIST OF [GRAND], [MAJOR], [MINOR] AND [MINI].</t>
+          <t>▪ THE BET CANNOT BE ADJUSTED AND THE REMAINING BUY FEATURE CANNOT BE CANCELLED BEFORE THE LAST BUY FEATURE IS COMPLETED.</t>
         </is>
       </c>
       <c r="H88" s="7" t="n"/>
@@ -2015,94 +2015,91 @@
     <row r="89">
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>▪ 選擇 {1} 個 [幣] 以揭示 [GRAND]、[MAJOR]、[MINOR] 或 [MINI]。</t>
+          <t>▪ 所有「購買特色」完成後，投注將切換回購買前的投注。</t>
         </is>
       </c>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="8" t="n"/>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>▪ SELECT A [COIN] TO REVEAL [GRAND], [MAJOR], [MINOR], OR [MINI].</t>
+          <t>▪ AFTER ALL BUY FEATURE ROUNDS ARE COMPLETED, THE BET WILL SWITCH BACK TO THE BET BEFORE THE PURCHASE.</t>
         </is>
       </c>
       <c r="H89" s="7" t="n"/>
       <c r="I89" s="8" t="n"/>
     </row>
-    <row r="90">
-      <c r="D90" s="6" t="inlineStr">
-        <is>
-          <t>▪ 當玩家獲得 {3} 個相同的 OP JACKPOT 特色符號，即可獲得該 OP JACKPOT 並結算總獎金。</t>
-        </is>
-      </c>
-      <c r="E90" s="7" t="n"/>
-      <c r="F90" s="8" t="n"/>
-      <c r="G90" s="6" t="inlineStr">
-        <is>
-          <t>▪ IF PLAYER GETS {3} SAME JACKPOT SYMBOLS WILL WIN THE JACKPOT AND CALCULATE TOTAL WINNINGS.</t>
-        </is>
-      </c>
-      <c r="H90" s="7" t="n"/>
-      <c r="I90" s="8" t="n"/>
-    </row>
     <row r="91">
-      <c r="D91" s="6" t="inlineStr">
-        <is>
-          <t>▪ [GRAND] 為連機累進彩金。單場遊戲中，投注選項選擇 {2.00} 以上即可解鎖 [GRAND]。</t>
-        </is>
-      </c>
-      <c r="E91" s="7" t="n"/>
-      <c r="F91" s="8" t="n"/>
-      <c r="G91" s="6" t="inlineStr">
-        <is>
-          <t>▪ [GRAND] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [GRAND].</t>
-        </is>
-      </c>
-      <c r="H91" s="7" t="n"/>
-      <c r="I91" s="8" t="n"/>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>OP JACKPOT</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>▪ [MAJOR] 為連機累進彩金。單場遊戲中，投注選項選擇 {2.00} 以上即可解鎖 [MAJOR]。</t>
-        </is>
-      </c>
-      <c r="E92" s="7" t="n"/>
-      <c r="F92" s="8" t="n"/>
-      <c r="G92" s="6" t="inlineStr">
-        <is>
-          <t>▪ [MAJOR] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [MAJOR].</t>
-        </is>
-      </c>
-      <c r="H92" s="7" t="n"/>
-      <c r="I92" s="8" t="n"/>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>繁中</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>英文</t>
+        </is>
+      </c>
     </row>
     <row r="93">
+      <c r="B93" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>主要標題</t>
+        </is>
+      </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>▪ [MINOR] 為紅利彩金，依照投注選項改變。</t>
+          <t>OP JACKPOT</t>
         </is>
       </c>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="8" t="n"/>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>▪ [MINOR] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
+          <t>OP JACKPOT</t>
         </is>
       </c>
       <c r="H93" s="7" t="n"/>
       <c r="I93" s="8" t="n"/>
     </row>
     <row r="94">
+      <c r="B94" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>規則說明</t>
+        </is>
+      </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>▪ [MINI] 為紅利彩金，依照投注選項改變。</t>
+          <t>▪ 在遊戲中，OP JACKPOT 特色由盤面上的 [C1] 隨機觸發。</t>
         </is>
       </c>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="8" t="n"/>
       <c r="G94" s="6" t="inlineStr">
         <is>
-          <t>▪ [MINI] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
+          <t>▪ OP JACKPOT FEATURE IS TRIGGERED RANDOMLY BY {1} OR MORE [C1] ON THE REELS.</t>
         </is>
       </c>
       <c r="H94" s="7" t="n"/>
@@ -2111,62 +2108,46 @@
     <row r="95">
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>▪ 玩家投注越高，觸發 OP JACKPOT 特色的機會越高。</t>
+          <t>▪ OP JACKPOT 特色會在畫面中出現 {12} 個 [幣]，其中包括 [GRAND]、[MAJOR]、[MINOR] 及 [MINI]。</t>
         </is>
       </c>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="8" t="n"/>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>▪ THE HIGHER BET, THE HIGHER CHANCES TO TRIGGER OP JACKPOT FEATURE.</t>
+          <t>▪ DURING OP JACKPOT FEATURE, THERE ARE {12} [COIN] WHICH CONSIST OF [GRAND], [MAJOR], [MINOR] AND [MINI].</t>
         </is>
       </c>
       <c r="H95" s="7" t="n"/>
       <c r="I95" s="8" t="n"/>
     </row>
     <row r="96">
-      <c r="B96" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>主要標題</t>
-        </is>
-      </c>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>OP JACKPOT</t>
+          <t>▪ 選擇 {1} 個 [幣] 以揭示 [GRAND]、[MAJOR]、[MINOR] 或 [MINI]。</t>
         </is>
       </c>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="8" t="n"/>
       <c r="G96" s="6" t="inlineStr">
         <is>
-          <t>OP JACKPOT</t>
+          <t>▪ SELECT A [COIN] TO REVEAL [GRAND], [MAJOR], [MINOR], OR [MINI].</t>
         </is>
       </c>
       <c r="H96" s="7" t="n"/>
       <c r="I96" s="8" t="n"/>
     </row>
     <row r="97">
-      <c r="B97" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t>規則說明</t>
-        </is>
-      </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>在游戏中，OP JACKPOT 特色由特色转轮上 [C1] 随机触发。</t>
+          <t>▪ 當玩家獲得 {3} 個相同的 OP JACKPOT 特色符號，即可獲得該 OP JACKPOT 並結算總獎金。</t>
         </is>
       </c>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="8" t="n"/>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>OP JACKPOT FEATURE IS TRIGGERED RANDOMLY BY {1} OR MORE [C1] ON THE REELS.</t>
+          <t>▪ IF PLAYER GETS {3} SAME JACKPOT SYMBOLS WILL WIN THE JACKPOT AND CALCULATE TOTAL WINNINGS.</t>
         </is>
       </c>
       <c r="H97" s="7" t="n"/>
@@ -2175,14 +2156,14 @@
     <row r="98">
       <c r="D98" s="6" t="inlineStr">
         <is>
-          <t>OP JACKPOT 特色会在画面中出现 {12} 个 [幣]，其中包括 [GRAND]、[MAJOR]、[MINOR] 及 [MINI]。</t>
+          <t>▪ [GRAND] 為連機累進彩金。單場遊戲中，投注選項選擇 {2.00} 以上即可解鎖 [GRAND]。</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="8" t="n"/>
       <c r="G98" s="6" t="inlineStr">
         <is>
-          <t>DURING OP JACKPOT FEATURE, THERE ARE {12} [COIN] WHICH CONSIST OF [GRAND], [MAJOR], [MINOR] AND [MINI].</t>
+          <t>▪ [GRAND] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [GRAND].</t>
         </is>
       </c>
       <c r="H98" s="7" t="n"/>
@@ -2191,14 +2172,14 @@
     <row r="99">
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>选择 {1} 个 [幣] 以揭示 [GRAND]、[MAJOR]、[MINOR] 或 [MINI]。</t>
+          <t>▪ [MAJOR] 為連機累進彩金。單場遊戲中，投注選項選擇 {2.00} 以上即可解鎖 [MAJOR]。</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="8" t="n"/>
       <c r="G99" s="6" t="inlineStr">
         <is>
-          <t>SELECT A [COIN] TO REVEAL [GRAND], [MAJOR], [MINOR], OR [MINI].</t>
+          <t>▪ [MAJOR] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [MAJOR].</t>
         </is>
       </c>
       <c r="H99" s="7" t="n"/>
@@ -2207,14 +2188,14 @@
     <row r="100">
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>当玩家获得 {3} 个相同的 OP JACKPOT 特色符号即可获得该 OP JACKPOT 并结算总奖金。</t>
+          <t>▪ [MINOR] 為紅利彩金，依照投注選項改變。</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="8" t="n"/>
       <c r="G100" s="6" t="inlineStr">
         <is>
-          <t>IF PLAYER GETS {3} SAME JACKPOT SYMBOLS WILL WIN THE JACKPOT AND CALCULATE TOTAL WINNINGS.</t>
+          <t>▪ [MINOR] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
         </is>
       </c>
       <c r="H100" s="7" t="n"/>
@@ -2223,14 +2204,14 @@
     <row r="101">
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>[GRAND] 为连机累进彩金。单场游戏中，投注选项选择 {2.00} 以上即可解锁 [GRAND]。</t>
+          <t>▪ [MINI] 為紅利彩金，依照投注選項改變。</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
       <c r="F101" s="8" t="n"/>
       <c r="G101" s="6" t="inlineStr">
         <is>
-          <t>[GRAND] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [GRAND].</t>
+          <t>▪ [MINI] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
         </is>
       </c>
       <c r="H101" s="7" t="n"/>
@@ -2239,46 +2220,62 @@
     <row r="102">
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>[MAJOR] 为连机累进彩金。单场游戏中，投注选项选择 {2.00} 以上即可解锁 [MAJOR]。</t>
+          <t>▪ 玩家投注越高，觸發 OP JACKPOT 特色的機會越高。</t>
         </is>
       </c>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="8" t="n"/>
       <c r="G102" s="6" t="inlineStr">
         <is>
-          <t>[MAJOR] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [MAJOR].</t>
+          <t>▪ THE HIGHER BET, THE HIGHER CHANCES TO TRIGGER OP JACKPOT FEATURE.</t>
         </is>
       </c>
       <c r="H102" s="7" t="n"/>
       <c r="I102" s="8" t="n"/>
     </row>
     <row r="103">
+      <c r="B103" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>主要標題</t>
+        </is>
+      </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>[MINOR] 为红利彩金，依照投注选项改变。</t>
+          <t>OP JACKPOT</t>
         </is>
       </c>
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="8" t="n"/>
       <c r="G103" s="6" t="inlineStr">
         <is>
-          <t>[MINOR] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
+          <t>OP JACKPOT</t>
         </is>
       </c>
       <c r="H103" s="7" t="n"/>
       <c r="I103" s="8" t="n"/>
     </row>
     <row r="104">
+      <c r="B104" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>規則說明</t>
+        </is>
+      </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>[MINI] 为红利彩金，依照投注选项改变。</t>
+          <t>在游戏中，OP JACKPOT 特色由特色转轮上 [C1] 随机触发。</t>
         </is>
       </c>
       <c r="E104" s="7" t="n"/>
       <c r="F104" s="8" t="n"/>
       <c r="G104" s="6" t="inlineStr">
         <is>
-          <t>[MINI] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
+          <t>OP JACKPOT FEATURE IS TRIGGERED RANDOMLY BY {1} OR MORE [C1] ON THE REELS.</t>
         </is>
       </c>
       <c r="H104" s="7" t="n"/>
@@ -2287,91 +2284,94 @@
     <row r="105">
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>玩家投注越高触发 OP JACKPOT 特色的机会越高。</t>
+          <t>OP JACKPOT 特色会在画面中出现 {12} 个 [幣]，其中包括 [GRAND]、[MAJOR]、[MINOR] 及 [MINI]。</t>
         </is>
       </c>
       <c r="E105" s="7" t="n"/>
       <c r="F105" s="8" t="n"/>
       <c r="G105" s="6" t="inlineStr">
         <is>
-          <t>THE HIGHER BET, THE HIGHER CHANCES TO TRIGGER OP JACKPOT FEATURE.</t>
+          <t>DURING OP JACKPOT FEATURE, THERE ARE {12} [COIN] WHICH CONSIST OF [GRAND], [MAJOR], [MINOR] AND [MINI].</t>
         </is>
       </c>
       <c r="H105" s="7" t="n"/>
       <c r="I105" s="8" t="n"/>
     </row>
+    <row r="106">
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t>选择 {1} 个 [幣] 以揭示 [GRAND]、[MAJOR]、[MINOR] 或 [MINI]。</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="n"/>
+      <c r="F106" s="8" t="n"/>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t>SELECT A [COIN] TO REVEAL [GRAND], [MAJOR], [MINOR], OR [MINI].</t>
+        </is>
+      </c>
+      <c r="H106" s="7" t="n"/>
+      <c r="I106" s="8" t="n"/>
+    </row>
     <row r="107">
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>LINES / WAYS</t>
-        </is>
-      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>当玩家获得 {3} 个相同的 OP JACKPOT 特色符号即可获得该 OP JACKPOT 并结算总奖金。</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="n"/>
+      <c r="F107" s="8" t="n"/>
+      <c r="G107" s="6" t="inlineStr">
+        <is>
+          <t>IF PLAYER GETS {3} SAME JACKPOT SYMBOLS WILL WIN THE JACKPOT AND CALCULATE TOTAL WINNINGS.</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="n"/>
+      <c r="I107" s="8" t="n"/>
     </row>
     <row r="108">
-      <c r="B108" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C108" s="4" t="inlineStr">
-        <is>
-          <t>項目</t>
-        </is>
-      </c>
-      <c r="D108" s="5" t="inlineStr">
-        <is>
-          <t>繁中</t>
-        </is>
-      </c>
-      <c r="G108" s="5" t="inlineStr">
-        <is>
-          <t>英文</t>
-        </is>
-      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>[GRAND] 为连机累进彩金。单场游戏中，投注选项选择 {2.00} 以上即可解锁 [GRAND]。</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n"/>
+      <c r="F108" s="8" t="n"/>
+      <c r="G108" s="6" t="inlineStr">
+        <is>
+          <t>[GRAND] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [GRAND].</t>
+        </is>
+      </c>
+      <c r="H108" s="7" t="n"/>
+      <c r="I108" s="8" t="n"/>
     </row>
     <row r="109">
-      <c r="B109" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C109" s="6" t="inlineStr">
-        <is>
-          <t>主要標題</t>
-        </is>
-      </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>最多路數</t>
+          <t>[MAJOR] 为连机累进彩金。单场游戏中，投注选项选择 {2.00} 以上即可解锁 [MAJOR]。</t>
         </is>
       </c>
       <c r="E109" s="7" t="n"/>
       <c r="F109" s="8" t="n"/>
       <c r="G109" s="6" t="inlineStr">
         <is>
-          <t>MAXIMUM WAYS</t>
+          <t>[MAJOR] IS LINKED PROGRESSIVE JACKPOT. IF THE SINGLE GAME BET OPTION IS {2.00} OR ABOVE, THE PLAYER WILL UNLOCK [MAJOR].</t>
         </is>
       </c>
       <c r="H109" s="7" t="n"/>
       <c r="I109" s="8" t="n"/>
     </row>
     <row r="110">
-      <c r="B110" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C110" s="6" t="inlineStr">
-        <is>
-          <t>規則說明</t>
-        </is>
-      </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>▪ 所有符號必須由最左至右連續出現，方可獲獎。</t>
+          <t>[MINOR] 为红利彩金，依照投注选项改变。</t>
         </is>
       </c>
       <c r="E110" s="7" t="n"/>
       <c r="F110" s="8" t="n"/>
       <c r="G110" s="6" t="inlineStr">
         <is>
-          <t>▪ ALL WINS ARE FROM LEFTMOST TO RIGHT ONLY.</t>
+          <t>[MINOR] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
         </is>
       </c>
       <c r="H110" s="7" t="n"/>
@@ -2380,14 +2380,14 @@
     <row r="111">
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>▪ 當同一路有多種獲獎組合，僅會賠付最高的獲獎組合。</t>
+          <t>[MINI] 为红利彩金，依照投注选项改变。</t>
         </is>
       </c>
       <c r="E111" s="7" t="n"/>
       <c r="F111" s="8" t="n"/>
       <c r="G111" s="6" t="inlineStr">
         <is>
-          <t>▪ ONLY THE HIGHEST WIN IS PAID WHEN THERE IS MORE THAN ONE WINNING COMBINATION WITH A CERTAIN SYMBOL.</t>
+          <t>[MINI] WILL CHANGE IF THE PLAYER SELECTS DIFFERENT BET OPTION.</t>
         </is>
       </c>
       <c r="H111" s="7" t="n"/>
@@ -2396,139 +2396,139 @@
     <row r="112">
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>▪ 遊戲設定 = 最多 {1,024} 路。</t>
+          <t>玩家投注越高触发 OP JACKPOT 特色的机会越高。</t>
         </is>
       </c>
       <c r="E112" s="7" t="n"/>
       <c r="F112" s="8" t="n"/>
       <c r="G112" s="6" t="inlineStr">
         <is>
-          <t>▪ GAME SETTING = {1,024} MAXIMUM WAYS.</t>
+          <t>THE HIGHER BET, THE HIGHER CHANCES TO TRIGGER OP JACKPOT FEATURE.</t>
         </is>
       </c>
       <c r="H112" s="7" t="n"/>
       <c r="I112" s="8" t="n"/>
     </row>
-    <row r="113">
-      <c r="D113" s="6" t="inlineStr">
-        <is>
-          <t>[走線圖- 1,024 MAX WAYS]</t>
-        </is>
-      </c>
-      <c r="E113" s="7" t="n"/>
-      <c r="F113" s="8" t="n"/>
-      <c r="G113" s="6" t="inlineStr">
-        <is>
-          <t>[走線圖- 1,024 MAX WAYS]</t>
-        </is>
-      </c>
-      <c r="H113" s="7" t="n"/>
-      <c r="I113" s="8" t="n"/>
-    </row>
     <row r="114">
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>[走線圖-3 OF A KIND PAYS 2 WAYS]</t>
-        </is>
-      </c>
-      <c r="E114" s="7" t="n"/>
-      <c r="F114" s="8" t="n"/>
-      <c r="G114" s="6" t="inlineStr">
-        <is>
-          <t>[走線圖-3 OF A KIND PAYS 2 WAYS]</t>
-        </is>
-      </c>
-      <c r="H114" s="7" t="n"/>
-      <c r="I114" s="8" t="n"/>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>LINES / WAYS</t>
+        </is>
+      </c>
     </row>
     <row r="115">
-      <c r="D115" s="6" t="inlineStr">
-        <is>
-          <t>[走線圖-NO WIN]</t>
-        </is>
-      </c>
-      <c r="E115" s="7" t="n"/>
-      <c r="F115" s="8" t="n"/>
-      <c r="G115" s="6" t="inlineStr">
-        <is>
-          <t>[走線圖-NO WIN]</t>
-        </is>
-      </c>
-      <c r="H115" s="7" t="n"/>
-      <c r="I115" s="8" t="n"/>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>繁中</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>英文</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>主要標題</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>最多路數</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="n"/>
+      <c r="F116" s="8" t="n"/>
+      <c r="G116" s="6" t="inlineStr">
+        <is>
+          <t>MAXIMUM WAYS</t>
+        </is>
+      </c>
+      <c r="H116" s="7" t="n"/>
+      <c r="I116" s="8" t="n"/>
     </row>
     <row r="117">
-      <c r="B117" s="3" t="inlineStr">
-        <is>
-          <t>GAME RULE</t>
-        </is>
-      </c>
+      <c r="B117" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C117" s="6" t="inlineStr">
+        <is>
+          <t>規則說明</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>▪ 所有符號必須由最左至右連續出現，方可獲獎。</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="n"/>
+      <c r="F117" s="8" t="n"/>
+      <c r="G117" s="6" t="inlineStr">
+        <is>
+          <t>▪ ALL WINS ARE FROM LEFTMOST TO RIGHT ONLY.</t>
+        </is>
+      </c>
+      <c r="H117" s="7" t="n"/>
+      <c r="I117" s="8" t="n"/>
     </row>
     <row r="118">
-      <c r="B118" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C118" s="4" t="inlineStr">
-        <is>
-          <t>項目</t>
-        </is>
-      </c>
-      <c r="D118" s="5" t="inlineStr">
-        <is>
-          <t>繁中</t>
-        </is>
-      </c>
-      <c r="G118" s="5" t="inlineStr">
-        <is>
-          <t>英文</t>
-        </is>
-      </c>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t>▪ 當同一路有多種獲獎組合，僅會賠付最高的獲獎組合。</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="n"/>
+      <c r="F118" s="8" t="n"/>
+      <c r="G118" s="6" t="inlineStr">
+        <is>
+          <t>▪ ONLY THE HIGHEST WIN IS PAID WHEN THERE IS MORE THAN ONE WINNING COMBINATION WITH A CERTAIN SYMBOL.</t>
+        </is>
+      </c>
+      <c r="H118" s="7" t="n"/>
+      <c r="I118" s="8" t="n"/>
     </row>
     <row r="119">
-      <c r="B119" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C119" s="6" t="inlineStr">
-        <is>
-          <t>主要標題</t>
-        </is>
-      </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>遊戲規則</t>
+          <t>▪ 遊戲設定 = 最多 {1,024} 路。</t>
         </is>
       </c>
       <c r="E119" s="7" t="n"/>
       <c r="F119" s="8" t="n"/>
       <c r="G119" s="6" t="inlineStr">
         <is>
-          <t>GAME RULES</t>
+          <t>▪ GAME SETTING = {1,024} MAXIMUM WAYS.</t>
         </is>
       </c>
       <c r="H119" s="7" t="n"/>
       <c r="I119" s="8" t="n"/>
     </row>
     <row r="120">
-      <c r="B120" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C120" s="6" t="inlineStr">
-        <is>
-          <t>規則說明</t>
-        </is>
-      </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>▪ 選擇您想要玩的投注選項。</t>
+          <t>[走線圖- 1,024 MAX WAYS]</t>
         </is>
       </c>
       <c r="E120" s="7" t="n"/>
       <c r="F120" s="8" t="n"/>
       <c r="G120" s="6" t="inlineStr">
         <is>
-          <t>▪ SELECT BET OPTION YOU WISH TO PLAY.</t>
+          <t>[走線圖- 1,024 MAX WAYS]</t>
         </is>
       </c>
       <c r="H120" s="7" t="n"/>
@@ -2537,14 +2537,14 @@
     <row r="121">
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>▪ 所有中獎金額均乘以投注選項，除非是累積獎。</t>
+          <t>[走線圖-3 OF A KIND PAYS 2 WAYS]</t>
         </is>
       </c>
       <c r="E121" s="7" t="n"/>
       <c r="F121" s="8" t="n"/>
       <c r="G121" s="6" t="inlineStr">
         <is>
-          <t>▪ ALL WINS ARE MULTIPLIED BY BET OPTION EXCEPT PROGRESSIVES BONUSES.</t>
+          <t>[走線圖-3 OF A KIND PAYS 2 WAYS]</t>
         </is>
       </c>
       <c r="H121" s="7" t="n"/>
@@ -2553,46 +2553,157 @@
     <row r="122">
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>▪ 遊戲出現故障時，所有賠付與遊戲結果均視為無效。</t>
+          <t>[走線圖-NO WIN]</t>
         </is>
       </c>
       <c r="E122" s="7" t="n"/>
       <c r="F122" s="8" t="n"/>
       <c r="G122" s="6" t="inlineStr">
         <is>
-          <t>▪ MALFUNCTION VOIDS ALL PAYS AND PLAYS.</t>
+          <t>[走線圖-NO WIN]</t>
         </is>
       </c>
       <c r="H122" s="7" t="n"/>
       <c r="I122" s="8" t="n"/>
     </row>
-    <row r="123">
-      <c r="D123" s="6" t="inlineStr">
+    <row r="124">
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>GAME RULE</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>繁中</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>英文</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>主要標題</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>遊戲規則</t>
+        </is>
+      </c>
+      <c r="E126" s="7" t="n"/>
+      <c r="F126" s="8" t="n"/>
+      <c r="G126" s="6" t="inlineStr">
+        <is>
+          <t>GAME RULES</t>
+        </is>
+      </c>
+      <c r="H126" s="7" t="n"/>
+      <c r="I126" s="8" t="n"/>
+    </row>
+    <row r="127">
+      <c r="B127" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>規則說明</t>
+        </is>
+      </c>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t>▪ 選擇您想要玩的投注選項。</t>
+        </is>
+      </c>
+      <c r="E127" s="7" t="n"/>
+      <c r="F127" s="8" t="n"/>
+      <c r="G127" s="6" t="inlineStr">
+        <is>
+          <t>▪ SELECT BET OPTION YOU WISH TO PLAY.</t>
+        </is>
+      </c>
+      <c r="H127" s="7" t="n"/>
+      <c r="I127" s="8" t="n"/>
+    </row>
+    <row r="128">
+      <c r="D128" s="6" t="inlineStr">
+        <is>
+          <t>▪ 所有中獎金額均乘以投注選項，除非是累積獎。</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="n"/>
+      <c r="F128" s="8" t="n"/>
+      <c r="G128" s="6" t="inlineStr">
+        <is>
+          <t>▪ ALL WINS ARE MULTIPLIED BY BET OPTION EXCEPT PROGRESSIVES BONUSES.</t>
+        </is>
+      </c>
+      <c r="H128" s="7" t="n"/>
+      <c r="I128" s="8" t="n"/>
+    </row>
+    <row r="129">
+      <c r="D129" s="6" t="inlineStr">
+        <is>
+          <t>▪ 遊戲出現故障時，所有賠付與遊戲結果均視為無效。</t>
+        </is>
+      </c>
+      <c r="E129" s="7" t="n"/>
+      <c r="F129" s="8" t="n"/>
+      <c r="G129" s="6" t="inlineStr">
+        <is>
+          <t>▪ MALFUNCTION VOIDS ALL PAYS AND PLAYS.</t>
+        </is>
+      </c>
+      <c r="H129" s="7" t="n"/>
+      <c r="I129" s="8" t="n"/>
+    </row>
+    <row r="130">
+      <c r="D130" s="6" t="inlineStr">
         <is>
           <t>▪ 若玩家在免費遊戲期間中斷連線，系統將自動完成該局結算，並將中獎金額加入餘額。</t>
         </is>
       </c>
-      <c r="E123" s="7" t="n"/>
-      <c r="F123" s="8" t="n"/>
-      <c r="G123" s="6" t="inlineStr">
+      <c r="E130" s="7" t="n"/>
+      <c r="F130" s="8" t="n"/>
+      <c r="G130" s="6" t="inlineStr">
         <is>
           <t>▪ IF THE PLAYER LOSES CONNECTION DURING THE FREE GAME FEATURE, THE SYSTEM WILL COMPLETE THE RESULT AUTOMATICALLY AND ADD ANY WINNINGS TO THE BALANCE.</t>
         </is>
       </c>
-      <c r="H123" s="7" t="n"/>
-      <c r="I123" s="8" t="n"/>
+      <c r="H130" s="7" t="n"/>
+      <c r="I130" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="156">
+  <mergeCells count="164">
     <mergeCell ref="G38:I38"/>
     <mergeCell ref="G103:I103"/>
     <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D76:F76"/>
     <mergeCell ref="G112:I112"/>
     <mergeCell ref="G13:I13"/>
+    <mergeCell ref="D116:F116"/>
     <mergeCell ref="G62:I62"/>
+    <mergeCell ref="G118:I118"/>
     <mergeCell ref="D66:F66"/>
     <mergeCell ref="G87:I87"/>
+    <mergeCell ref="G127:I127"/>
     <mergeCell ref="D75:F75"/>
     <mergeCell ref="D53:F53"/>
     <mergeCell ref="D47:F47"/>
@@ -2607,17 +2718,18 @@
     <mergeCell ref="G73:I73"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="G88:I88"/>
-    <mergeCell ref="D92:F92"/>
     <mergeCell ref="D30:F30"/>
     <mergeCell ref="D39:F39"/>
+    <mergeCell ref="G129:I129"/>
     <mergeCell ref="G63:I63"/>
     <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G90:I90"/>
     <mergeCell ref="D94:F94"/>
+    <mergeCell ref="D129:F129"/>
     <mergeCell ref="G9:I9"/>
     <mergeCell ref="D119:F119"/>
-    <mergeCell ref="G115:I115"/>
     <mergeCell ref="G36:I36"/>
+    <mergeCell ref="D128:F128"/>
+    <mergeCell ref="G107:I107"/>
     <mergeCell ref="D80:F80"/>
     <mergeCell ref="D96:F96"/>
     <mergeCell ref="D105:F105"/>
@@ -2625,23 +2737,27 @@
     <mergeCell ref="G101:I101"/>
     <mergeCell ref="D120:F120"/>
     <mergeCell ref="G37:I37"/>
-    <mergeCell ref="G78:I78"/>
-    <mergeCell ref="D91:F91"/>
-    <mergeCell ref="G92:I92"/>
+    <mergeCell ref="D107:F107"/>
     <mergeCell ref="G30:I30"/>
     <mergeCell ref="G14:I14"/>
+    <mergeCell ref="D106:F106"/>
     <mergeCell ref="G80:I80"/>
     <mergeCell ref="D93:F93"/>
     <mergeCell ref="G55:I55"/>
     <mergeCell ref="G64:I64"/>
     <mergeCell ref="D74:F74"/>
+    <mergeCell ref="D130:F130"/>
     <mergeCell ref="D68:F68"/>
+    <mergeCell ref="D83:F83"/>
+    <mergeCell ref="D117:F117"/>
     <mergeCell ref="D55:F55"/>
     <mergeCell ref="G54:I54"/>
     <mergeCell ref="G119:I119"/>
     <mergeCell ref="G32:I32"/>
     <mergeCell ref="D67:F67"/>
     <mergeCell ref="D110:F110"/>
+    <mergeCell ref="D85:F85"/>
+    <mergeCell ref="G106:I106"/>
     <mergeCell ref="D54:F54"/>
     <mergeCell ref="D60:F60"/>
     <mergeCell ref="G56:I56"/>
@@ -2657,6 +2773,7 @@
     <mergeCell ref="D40:F40"/>
     <mergeCell ref="G8:I8"/>
     <mergeCell ref="D111:F111"/>
+    <mergeCell ref="D108:F108"/>
     <mergeCell ref="D86:F86"/>
     <mergeCell ref="G82:I82"/>
     <mergeCell ref="D95:F95"/>
@@ -2670,13 +2787,12 @@
     <mergeCell ref="G74:I74"/>
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="G68:I68"/>
-    <mergeCell ref="D78:F78"/>
+    <mergeCell ref="G83:I83"/>
     <mergeCell ref="D87:F87"/>
+    <mergeCell ref="G108:I108"/>
     <mergeCell ref="D122:F122"/>
-    <mergeCell ref="G123:I123"/>
     <mergeCell ref="G45:I45"/>
     <mergeCell ref="G110:I110"/>
-    <mergeCell ref="G113:I113"/>
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="D121:F121"/>
     <mergeCell ref="G100:I100"/>
@@ -2685,42 +2801,41 @@
     <mergeCell ref="G109:I109"/>
     <mergeCell ref="G47:I47"/>
     <mergeCell ref="D82:F82"/>
-    <mergeCell ref="D113:F113"/>
     <mergeCell ref="G44:I44"/>
+    <mergeCell ref="G84:I84"/>
     <mergeCell ref="G31:I31"/>
     <mergeCell ref="G46:I46"/>
     <mergeCell ref="G102:I102"/>
-    <mergeCell ref="D123:F123"/>
     <mergeCell ref="G40:I40"/>
     <mergeCell ref="G111:I111"/>
     <mergeCell ref="D44:F44"/>
     <mergeCell ref="G12:I12"/>
-    <mergeCell ref="D115:F115"/>
     <mergeCell ref="G72:I72"/>
     <mergeCell ref="G86:I86"/>
     <mergeCell ref="D99:F99"/>
+    <mergeCell ref="D84:F84"/>
     <mergeCell ref="D36:F36"/>
     <mergeCell ref="G97:I97"/>
     <mergeCell ref="D45:F45"/>
     <mergeCell ref="D101:F101"/>
     <mergeCell ref="G7:I7"/>
-    <mergeCell ref="D77:F77"/>
     <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G128:I128"/>
     <mergeCell ref="D61:F61"/>
+    <mergeCell ref="D126:F126"/>
     <mergeCell ref="D48:F48"/>
     <mergeCell ref="G49:I49"/>
     <mergeCell ref="G121:I121"/>
     <mergeCell ref="D72:F72"/>
     <mergeCell ref="D103:F103"/>
     <mergeCell ref="D112:F112"/>
-    <mergeCell ref="G114:I114"/>
     <mergeCell ref="D62:F62"/>
+    <mergeCell ref="D118:F118"/>
     <mergeCell ref="D56:F56"/>
-    <mergeCell ref="D114:F114"/>
-    <mergeCell ref="G76:I76"/>
-    <mergeCell ref="G91:I91"/>
+    <mergeCell ref="D127:F127"/>
     <mergeCell ref="D64:F64"/>
     <mergeCell ref="D38:F38"/>
+    <mergeCell ref="G85:I85"/>
     <mergeCell ref="D89:F89"/>
     <mergeCell ref="D98:F98"/>
     <mergeCell ref="G99:I99"/>
@@ -2728,17 +2843,19 @@
     <mergeCell ref="D79:F79"/>
     <mergeCell ref="G75:I75"/>
     <mergeCell ref="D88:F88"/>
+    <mergeCell ref="G130:I130"/>
     <mergeCell ref="D63:F63"/>
-    <mergeCell ref="G77:I77"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="D81:F81"/>
-    <mergeCell ref="D90:F90"/>
+    <mergeCell ref="G117:I117"/>
     <mergeCell ref="G67:I67"/>
     <mergeCell ref="D65:F65"/>
     <mergeCell ref="G61:I61"/>
+    <mergeCell ref="G126:I126"/>
     <mergeCell ref="G39:I39"/>
     <mergeCell ref="G48:I48"/>
+    <mergeCell ref="G116:I116"/>
     <mergeCell ref="D49:F49"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>